<commit_message>
tree 1 pattern completed
</commit_message>
<xml_diff>
--- a/LeetCode Patterns.xlsx
+++ b/LeetCode Patterns.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sksat\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\placements\practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D56097D-CF3B-45CB-863E-0205535D4F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31987ECD-CA1A-4507-8483-617A423B3E6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="485" uniqueCount="476">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="486" uniqueCount="477">
   <si>
     <t xml:space="preserve">Author : Taufique </t>
   </si>
@@ -1459,6 +1459,9 @@
   </si>
   <si>
     <t>COMP</t>
+  </si>
+  <si>
+    <t>striver</t>
   </si>
 </sst>
 </file>
@@ -1576,7 +1579,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1588,6 +1591,7 @@
     <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="6" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10204,6 +10208,9 @@
       <c r="AA12" s="4"/>
     </row>
     <row r="13" spans="1:27" ht="15.5" x14ac:dyDescent="0.35">
+      <c r="A13" s="11" t="s">
+        <v>476</v>
+      </c>
       <c r="B13" s="3" t="s">
         <v>12</v>
       </c>

</xml_diff>